<commit_message>
Sync revised animal balance table and isolate ordinary launcher
</commit_message>
<xml_diff>
--- a/单位属性表/20261010.xlsx
+++ b/单位属性表/20261010.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\cruelworld\Desktop\codex\奇境王冠\单位属性表\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{041126C3-98AD-4CE0-A5F1-993D62F08933}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7BD61D8F-51B9-4A91-A091-B41AEBF730D0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-93" yWindow="-93" windowWidth="25786" windowHeight="13986" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -944,6 +944,27 @@
     <xf numFmtId="0" fontId="2" fillId="13" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="17" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="9" fillId="9" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="12" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -953,15 +974,6 @@
     <xf numFmtId="0" fontId="7" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="13" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -973,18 +985,6 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="9" fillId="9" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1391,7 +1391,7 @@
         <v>80</v>
       </c>
       <c r="F2" s="2">
-        <v>60</v>
+        <v>40</v>
       </c>
       <c r="G2" s="2">
         <v>200</v>
@@ -1427,13 +1427,13 @@
         <v>700</v>
       </c>
       <c r="D3" s="2">
-        <v>30</v>
+        <v>25</v>
       </c>
       <c r="E3" s="2">
         <v>60</v>
       </c>
       <c r="F3" s="2">
-        <v>70</v>
+        <v>50</v>
       </c>
       <c r="G3" s="2">
         <v>500</v>
@@ -1455,7 +1455,7 @@
       </c>
       <c r="M3" s="6">
         <f>D3/G3*1000</f>
-        <v>60</v>
+        <v>50</v>
       </c>
     </row>
     <row r="4" spans="1:14" s="6" customFormat="1" ht="30.7">
@@ -1475,7 +1475,7 @@
         <v>40</v>
       </c>
       <c r="F4" s="2">
-        <v>80</v>
+        <v>60</v>
       </c>
       <c r="G4" s="2">
         <v>800</v>
@@ -1517,7 +1517,7 @@
         <v>50</v>
       </c>
       <c r="F5" s="2">
-        <v>100</v>
+        <v>80</v>
       </c>
       <c r="G5" s="2">
         <v>1000</v>
@@ -1546,15 +1546,15 @@
     <row r="7" spans="1:14" s="6" customFormat="1"/>
     <row r="8" spans="1:14" s="6" customFormat="1"/>
     <row r="9" spans="1:14" ht="28">
-      <c r="A9" s="17" t="s">
+      <c r="A9" s="24" t="s">
         <v>40</v>
       </c>
-      <c r="B9" s="17"/>
-      <c r="C9" s="17"/>
-      <c r="D9" s="17"/>
-      <c r="E9" s="17"/>
-      <c r="F9" s="17"/>
-      <c r="G9" s="17"/>
+      <c r="B9" s="24"/>
+      <c r="C9" s="24"/>
+      <c r="D9" s="24"/>
+      <c r="E9" s="24"/>
+      <c r="F9" s="24"/>
+      <c r="G9" s="24"/>
       <c r="H9" s="12"/>
       <c r="I9" s="12"/>
       <c r="J9" s="6"/>
@@ -1564,17 +1564,17 @@
       <c r="N9" s="6"/>
     </row>
     <row r="10" spans="1:14" ht="20">
-      <c r="A10" s="23" t="s">
+      <c r="A10" s="27" t="s">
         <v>41</v>
       </c>
-      <c r="B10" s="23"/>
-      <c r="C10" s="18">
+      <c r="B10" s="27"/>
+      <c r="C10" s="25">
         <v>5</v>
       </c>
-      <c r="D10" s="18"/>
-      <c r="E10" s="18"/>
-      <c r="F10" s="18"/>
-      <c r="G10" s="18"/>
+      <c r="D10" s="25"/>
+      <c r="E10" s="25"/>
+      <c r="F10" s="25"/>
+      <c r="G10" s="25"/>
       <c r="H10" s="13"/>
       <c r="I10" s="13"/>
       <c r="J10" s="6"/>
@@ -1584,17 +1584,17 @@
       <c r="N10" s="6"/>
     </row>
     <row r="11" spans="1:14" ht="19.350000000000001">
-      <c r="A11" s="19" t="s">
+      <c r="A11" s="26" t="s">
         <v>42</v>
       </c>
-      <c r="B11" s="19"/>
-      <c r="C11" s="19">
+      <c r="B11" s="26"/>
+      <c r="C11" s="26">
         <v>20</v>
       </c>
-      <c r="D11" s="19"/>
-      <c r="E11" s="19"/>
-      <c r="F11" s="19"/>
-      <c r="G11" s="19"/>
+      <c r="D11" s="26"/>
+      <c r="E11" s="26"/>
+      <c r="F11" s="26"/>
+      <c r="G11" s="26"/>
       <c r="H11" s="6"/>
       <c r="I11" s="6"/>
       <c r="J11" s="6"/>
@@ -1604,21 +1604,21 @@
       <c r="N11" s="6"/>
     </row>
     <row r="12" spans="1:14" ht="19.350000000000001">
-      <c r="A12" s="24" t="s">
+      <c r="A12" s="28" t="s">
         <v>43</v>
       </c>
-      <c r="B12" s="19"/>
-      <c r="C12" s="19">
+      <c r="B12" s="26"/>
+      <c r="C12" s="26">
         <v>30</v>
       </c>
-      <c r="D12" s="19"/>
-      <c r="E12" s="19"/>
-      <c r="F12" s="19"/>
-      <c r="G12" s="19"/>
-      <c r="H12" s="26" t="s">
+      <c r="D12" s="26"/>
+      <c r="E12" s="26"/>
+      <c r="F12" s="26"/>
+      <c r="G12" s="26"/>
+      <c r="H12" s="30" t="s">
         <v>62</v>
       </c>
-      <c r="I12" s="26"/>
+      <c r="I12" s="30"/>
       <c r="J12" s="6"/>
       <c r="K12" s="6"/>
       <c r="L12" s="6"/>
@@ -1674,7 +1674,7 @@
       <c r="F14" s="11">
         <v>1</v>
       </c>
-      <c r="G14" s="30" t="s">
+      <c r="G14" s="17" t="s">
         <v>63</v>
       </c>
     </row>
@@ -1850,16 +1850,16 @@
       <c r="N23" s="6"/>
     </row>
     <row r="24" spans="1:14" ht="35" customHeight="1">
-      <c r="A24" s="20" t="s">
+      <c r="A24" s="22" t="s">
         <v>31</v>
       </c>
-      <c r="B24" s="21"/>
-      <c r="C24" s="21"/>
-      <c r="D24" s="21"/>
-      <c r="E24" s="21"/>
+      <c r="B24" s="23"/>
+      <c r="C24" s="23"/>
+      <c r="D24" s="23"/>
+      <c r="E24" s="23"/>
       <c r="F24" s="16"/>
-      <c r="G24" s="25"/>
-      <c r="H24" s="25"/>
+      <c r="G24" s="29"/>
+      <c r="H24" s="29"/>
       <c r="I24" s="15"/>
       <c r="J24" s="6"/>
       <c r="K24" s="6"/>
@@ -1871,131 +1871,131 @@
       <c r="A25" s="3" t="s">
         <v>25</v>
       </c>
-      <c r="B25" s="22" t="s">
+      <c r="B25" s="18" t="s">
         <v>58</v>
       </c>
-      <c r="C25" s="22"/>
-      <c r="D25" s="22"/>
-      <c r="E25" s="22"/>
+      <c r="C25" s="18"/>
+      <c r="D25" s="18"/>
+      <c r="E25" s="18"/>
     </row>
     <row r="26" spans="1:14" s="6" customFormat="1" ht="16">
       <c r="A26" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="B26" s="22" t="s">
+      <c r="B26" s="18" t="s">
         <v>24</v>
       </c>
-      <c r="C26" s="22"/>
-      <c r="D26" s="22"/>
-      <c r="E26" s="22"/>
+      <c r="C26" s="18"/>
+      <c r="D26" s="18"/>
+      <c r="E26" s="18"/>
     </row>
     <row r="27" spans="1:14" s="6" customFormat="1" ht="16">
-      <c r="A27" s="22" t="s">
+      <c r="A27" s="18" t="s">
         <v>26</v>
       </c>
-      <c r="B27" s="22"/>
-      <c r="C27" s="22">
+      <c r="B27" s="18"/>
+      <c r="C27" s="18">
         <v>20</v>
       </c>
-      <c r="D27" s="22"/>
-      <c r="E27" s="22"/>
+      <c r="D27" s="18"/>
+      <c r="E27" s="18"/>
     </row>
     <row r="28" spans="1:14" s="6" customFormat="1" ht="16">
-      <c r="A28" s="22" t="s">
+      <c r="A28" s="18" t="s">
         <v>16</v>
       </c>
-      <c r="B28" s="22"/>
-      <c r="C28" s="22">
+      <c r="B28" s="18"/>
+      <c r="C28" s="18">
         <v>20</v>
       </c>
-      <c r="D28" s="22"/>
-      <c r="E28" s="22"/>
+      <c r="D28" s="18"/>
+      <c r="E28" s="18"/>
     </row>
     <row r="29" spans="1:14" s="6" customFormat="1" ht="16">
-      <c r="A29" s="22" t="s">
+      <c r="A29" s="18" t="s">
         <v>27</v>
       </c>
-      <c r="B29" s="22"/>
-      <c r="C29" s="22">
+      <c r="B29" s="18"/>
+      <c r="C29" s="18">
         <v>1000</v>
       </c>
-      <c r="D29" s="22"/>
-      <c r="E29" s="22"/>
+      <c r="D29" s="18"/>
+      <c r="E29" s="18"/>
     </row>
     <row r="30" spans="1:14" s="6" customFormat="1" ht="28">
-      <c r="A30" s="20" t="s">
+      <c r="A30" s="22" t="s">
         <v>32</v>
       </c>
-      <c r="B30" s="21"/>
-      <c r="C30" s="21"/>
-      <c r="D30" s="21"/>
-      <c r="E30" s="21"/>
+      <c r="B30" s="23"/>
+      <c r="C30" s="23"/>
+      <c r="D30" s="23"/>
+      <c r="E30" s="23"/>
     </row>
     <row r="31" spans="1:14" s="6" customFormat="1" ht="16">
       <c r="A31" s="3" t="s">
         <v>25</v>
       </c>
-      <c r="B31" s="22" t="s">
+      <c r="B31" s="18" t="s">
         <v>33</v>
       </c>
-      <c r="C31" s="22"/>
-      <c r="D31" s="22"/>
-      <c r="E31" s="22"/>
+      <c r="C31" s="18"/>
+      <c r="D31" s="18"/>
+      <c r="E31" s="18"/>
     </row>
     <row r="32" spans="1:14" s="6" customFormat="1" ht="16">
       <c r="A32" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="B32" s="22" t="s">
+      <c r="B32" s="18" t="s">
         <v>34</v>
       </c>
-      <c r="C32" s="22"/>
-      <c r="D32" s="22"/>
-      <c r="E32" s="22"/>
+      <c r="C32" s="18"/>
+      <c r="D32" s="18"/>
+      <c r="E32" s="18"/>
     </row>
     <row r="33" spans="1:5" s="6" customFormat="1" ht="16">
-      <c r="A33" s="22" t="s">
+      <c r="A33" s="18" t="s">
         <v>35</v>
       </c>
-      <c r="B33" s="22"/>
-      <c r="C33" s="22">
+      <c r="B33" s="18"/>
+      <c r="C33" s="18">
         <v>2000</v>
       </c>
-      <c r="D33" s="22"/>
-      <c r="E33" s="22"/>
+      <c r="D33" s="18"/>
+      <c r="E33" s="18"/>
     </row>
     <row r="34" spans="1:5" s="6" customFormat="1" ht="16">
-      <c r="A34" s="22" t="s">
+      <c r="A34" s="18" t="s">
         <v>27</v>
       </c>
-      <c r="B34" s="22"/>
-      <c r="C34" s="22">
+      <c r="B34" s="18"/>
+      <c r="C34" s="18">
         <v>150</v>
       </c>
-      <c r="D34" s="22"/>
-      <c r="E34" s="22"/>
+      <c r="D34" s="18"/>
+      <c r="E34" s="18"/>
     </row>
     <row r="35" spans="1:5" s="6" customFormat="1" ht="44" customHeight="1">
-      <c r="A35" s="27" t="s">
+      <c r="A35" s="19" t="s">
         <v>36</v>
       </c>
-      <c r="B35" s="27"/>
-      <c r="C35" s="28" t="s">
+      <c r="B35" s="19"/>
+      <c r="C35" s="20" t="s">
         <v>59</v>
       </c>
-      <c r="D35" s="28"/>
-      <c r="E35" s="28"/>
+      <c r="D35" s="20"/>
+      <c r="E35" s="20"/>
     </row>
     <row r="36" spans="1:5" s="6" customFormat="1">
-      <c r="A36" s="29" t="s">
+      <c r="A36" s="21" t="s">
         <v>17</v>
       </c>
-      <c r="B36" s="29"/>
-      <c r="C36" s="29" t="s">
+      <c r="B36" s="21"/>
+      <c r="C36" s="21" t="s">
         <v>18</v>
       </c>
-      <c r="D36" s="29"/>
-      <c r="E36" s="29"/>
+      <c r="D36" s="21"/>
+      <c r="E36" s="21"/>
     </row>
     <row r="37" spans="1:5" s="6" customFormat="1"/>
     <row r="38" spans="1:5" s="6" customFormat="1"/>
@@ -2015,23 +2015,6 @@
     <row r="52" s="6" customFormat="1"/>
   </sheetData>
   <mergeCells count="29">
-    <mergeCell ref="A34:B34"/>
-    <mergeCell ref="C34:E34"/>
-    <mergeCell ref="A35:B35"/>
-    <mergeCell ref="C35:E35"/>
-    <mergeCell ref="A36:B36"/>
-    <mergeCell ref="C36:E36"/>
-    <mergeCell ref="A30:E30"/>
-    <mergeCell ref="B31:E31"/>
-    <mergeCell ref="B32:E32"/>
-    <mergeCell ref="A33:B33"/>
-    <mergeCell ref="C33:E33"/>
-    <mergeCell ref="A28:B28"/>
-    <mergeCell ref="C28:E28"/>
-    <mergeCell ref="A29:B29"/>
-    <mergeCell ref="C29:E29"/>
-    <mergeCell ref="B25:E25"/>
-    <mergeCell ref="B26:E26"/>
     <mergeCell ref="A9:G9"/>
     <mergeCell ref="C10:G10"/>
     <mergeCell ref="C11:G11"/>
@@ -2044,6 +2027,23 @@
     <mergeCell ref="C12:G12"/>
     <mergeCell ref="G24:H24"/>
     <mergeCell ref="H12:I12"/>
+    <mergeCell ref="A28:B28"/>
+    <mergeCell ref="C28:E28"/>
+    <mergeCell ref="A29:B29"/>
+    <mergeCell ref="C29:E29"/>
+    <mergeCell ref="B25:E25"/>
+    <mergeCell ref="B26:E26"/>
+    <mergeCell ref="A30:E30"/>
+    <mergeCell ref="B31:E31"/>
+    <mergeCell ref="B32:E32"/>
+    <mergeCell ref="A33:B33"/>
+    <mergeCell ref="C33:E33"/>
+    <mergeCell ref="A34:B34"/>
+    <mergeCell ref="C34:E34"/>
+    <mergeCell ref="A35:B35"/>
+    <mergeCell ref="C35:E35"/>
+    <mergeCell ref="A36:B36"/>
+    <mergeCell ref="C36:E36"/>
   </mergeCells>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>